<commit_message>
#42 BOM updated with R12 removed from DNP.
</commit_message>
<xml_diff>
--- a/Design Files/Smart-Speaker-v2.1/BOM/Client_BOM_IoT-Speaker-v2.1.xlsx
+++ b/Design Files/Smart-Speaker-v2.1/BOM/Client_BOM_IoT-Speaker-v2.1.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="459" uniqueCount="286">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="458" uniqueCount="286">
   <si>
     <t>#</t>
   </si>
@@ -611,6 +611,9 @@
     <t>RC0603JR-070RL</t>
   </si>
   <si>
+    <t>0R</t>
+  </si>
+  <si>
     <t>R13</t>
   </si>
   <si>
@@ -636,9 +639,6 @@
   </si>
   <si>
     <t>R16</t>
-  </si>
-  <si>
-    <t>0R</t>
   </si>
   <si>
     <t>R17, R18, R19, R20, R21, R22</t>
@@ -949,6 +949,13 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <strike/>
       <sz val="9"/>
@@ -971,13 +978,6 @@
       <color rgb="FF800080"/>
       <name val="Calibri"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1574,28 +1574,28 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="13" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1719,7 +1719,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1756,6 +1756,9 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1771,16 +1774,16 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="7" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="12" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="12" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2132,9 +2135,9 @@
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
       <c r="H1" s="4"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19"/>
     </row>
     <row r="2" ht="15.75" spans="1:11">
       <c r="A2" s="2"/>
@@ -3191,7 +3194,7 @@
       <c r="J34" s="12">
         <v>2</v>
       </c>
-      <c r="K34" s="19" t="s">
+      <c r="K34" s="20" t="s">
         <v>163</v>
       </c>
     </row>
@@ -3225,7 +3228,7 @@
       <c r="J35" s="13">
         <v>1</v>
       </c>
-      <c r="K35" s="19" t="s">
+      <c r="K35" s="20" t="s">
         <v>163</v>
       </c>
     </row>
@@ -3357,7 +3360,7 @@
       </c>
       <c r="K39" s="9"/>
     </row>
-    <row r="40" ht="15.75" spans="1:11">
+    <row r="40" spans="1:11">
       <c r="A40" s="2"/>
       <c r="B40" s="7">
         <f t="shared" si="0"/>
@@ -3389,7 +3392,7 @@
       </c>
       <c r="K40" s="11"/>
     </row>
-    <row r="41" ht="15.75" spans="1:11">
+    <row r="41" spans="1:11">
       <c r="A41" s="2"/>
       <c r="B41" s="7">
         <f t="shared" si="0"/>
@@ -3398,32 +3401,30 @@
       <c r="C41" s="8" t="s">
         <v>152</v>
       </c>
-      <c r="D41" s="12" t="s">
+      <c r="D41" s="14" t="s">
         <v>191</v>
       </c>
-      <c r="E41" s="12" t="s">
+      <c r="E41" s="14" t="s">
         <v>192</v>
       </c>
-      <c r="F41" s="12" t="s">
+      <c r="F41" s="14" t="s">
         <v>155</v>
       </c>
-      <c r="G41" s="12" t="s">
+      <c r="G41" s="14" t="s">
         <v>193</v>
       </c>
-      <c r="H41" s="12" t="s">
+      <c r="H41" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="I41" s="12" t="s">
-        <v>162</v>
-      </c>
-      <c r="J41" s="12">
+      <c r="I41" s="14" t="s">
+        <v>194</v>
+      </c>
+      <c r="J41" s="14">
         <v>1</v>
       </c>
-      <c r="K41" s="19" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="42" ht="15.75" spans="1:11">
+      <c r="K41" s="20"/>
+    </row>
+    <row r="42" spans="1:11">
       <c r="A42" s="2"/>
       <c r="B42" s="7">
         <f t="shared" si="0"/>
@@ -3433,22 +3434,22 @@
         <v>152</v>
       </c>
       <c r="D42" s="11" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E42" s="11" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="F42" s="11" t="s">
         <v>184</v>
       </c>
       <c r="G42" s="11" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="H42" s="11" t="s">
         <v>15</v>
       </c>
       <c r="I42" s="11" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="J42" s="11">
         <v>1</v>
@@ -3465,16 +3466,16 @@
         <v>164</v>
       </c>
       <c r="D43" s="12" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="E43" s="12" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="F43" s="12" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="G43" s="12" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="H43" s="12" t="s">
         <v>15</v>
@@ -3485,7 +3486,7 @@
       <c r="J43" s="12">
         <v>3</v>
       </c>
-      <c r="K43" s="19" t="s">
+      <c r="K43" s="20" t="s">
         <v>163</v>
       </c>
     </row>
@@ -3499,22 +3500,22 @@
         <v>164</v>
       </c>
       <c r="D44" s="11" t="s">
+        <v>203</v>
+      </c>
+      <c r="E44" s="11" t="s">
+        <v>200</v>
+      </c>
+      <c r="F44" s="11" t="s">
+        <v>201</v>
+      </c>
+      <c r="G44" s="11" t="s">
         <v>202</v>
-      </c>
-      <c r="E44" s="11" t="s">
-        <v>199</v>
-      </c>
-      <c r="F44" s="11" t="s">
-        <v>200</v>
-      </c>
-      <c r="G44" s="11" t="s">
-        <v>201</v>
       </c>
       <c r="H44" s="11" t="s">
         <v>15</v>
       </c>
       <c r="I44" s="11" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="J44" s="11">
         <v>1</v>
@@ -3610,7 +3611,7 @@
         <v>15</v>
       </c>
       <c r="I47" s="9" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="J47" s="9">
         <v>1</v>
@@ -3647,7 +3648,7 @@
       <c r="J48" s="12">
         <v>4</v>
       </c>
-      <c r="K48" s="19" t="s">
+      <c r="K48" s="20" t="s">
         <v>163</v>
       </c>
     </row>
@@ -3676,7 +3677,7 @@
         <v>15</v>
       </c>
       <c r="I49" s="9" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="J49" s="9">
         <v>2</v>
@@ -3713,7 +3714,7 @@
       <c r="J50" s="12">
         <v>1</v>
       </c>
-      <c r="K50" s="19" t="s">
+      <c r="K50" s="20" t="s">
         <v>163</v>
       </c>
     </row>
@@ -4103,42 +4104,42 @@
     </row>
     <row r="63" ht="24.75" spans="1:11">
       <c r="A63" s="2"/>
-      <c r="B63" s="14">
+      <c r="B63" s="15">
         <f t="shared" si="0"/>
         <v>61</v>
       </c>
-      <c r="C63" s="15" t="s">
+      <c r="C63" s="16" t="s">
         <v>275</v>
       </c>
-      <c r="D63" s="16" t="s">
+      <c r="D63" s="17" t="s">
         <v>276</v>
       </c>
-      <c r="E63" s="16" t="s">
+      <c r="E63" s="17" t="s">
         <v>277</v>
       </c>
-      <c r="F63" s="16" t="s">
+      <c r="F63" s="17" t="s">
         <v>278</v>
       </c>
-      <c r="G63" s="16" t="s">
+      <c r="G63" s="17" t="s">
         <v>279</v>
       </c>
-      <c r="H63" s="16" t="s">
+      <c r="H63" s="17" t="s">
         <v>280</v>
       </c>
-      <c r="I63" s="16" t="s">
+      <c r="I63" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="J63" s="16">
+      <c r="J63" s="17">
         <v>1</v>
       </c>
-      <c r="K63" s="16"/>
+      <c r="K63" s="17"/>
     </row>
     <row r="64" ht="48.75" spans="1:11">
       <c r="A64" s="2"/>
-      <c r="B64" s="14">
+      <c r="B64" s="15">
         <v>62</v>
       </c>
-      <c r="C64" s="17" t="s">
+      <c r="C64" s="18" t="s">
         <v>281</v>
       </c>
       <c r="D64" s="11" t="s">
@@ -4162,40 +4163,40 @@
       <c r="J64" s="11">
         <v>1</v>
       </c>
-      <c r="K64" s="20" t="s">
+      <c r="K64" s="21" t="s">
         <v>283</v>
       </c>
     </row>
     <row r="65" ht="48.75" spans="1:11">
       <c r="A65" s="2"/>
-      <c r="B65" s="14">
+      <c r="B65" s="15">
         <v>63</v>
       </c>
-      <c r="C65" s="17" t="s">
+      <c r="C65" s="18" t="s">
         <v>284</v>
       </c>
-      <c r="D65" s="21" t="s">
+      <c r="D65" s="22" t="s">
         <v>90</v>
       </c>
-      <c r="E65" s="21" t="s">
+      <c r="E65" s="22" t="s">
         <v>282</v>
       </c>
-      <c r="F65" s="21" t="s">
+      <c r="F65" s="22" t="s">
         <v>90</v>
       </c>
-      <c r="G65" s="21" t="s">
+      <c r="G65" s="22" t="s">
         <v>90</v>
       </c>
-      <c r="H65" s="21" t="s">
+      <c r="H65" s="22" t="s">
         <v>90</v>
       </c>
-      <c r="I65" s="21" t="s">
+      <c r="I65" s="22" t="s">
         <v>90</v>
       </c>
-      <c r="J65" s="21">
+      <c r="J65" s="22">
         <v>1</v>
       </c>
-      <c r="K65" s="22" t="s">
+      <c r="K65" s="23" t="s">
         <v>285</v>
       </c>
     </row>

</xml_diff>

<commit_message>
#42 MOD: Speaker added for Reference in Client BOM - Speaker Board
</commit_message>
<xml_diff>
--- a/Design Files/Smart-Speaker-v2.1/BOM/Client_BOM_IoT-Speaker-v2.1.xlsx
+++ b/Design Files/Smart-Speaker-v2.1/BOM/Client_BOM_IoT-Speaker-v2.1.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="458" uniqueCount="286">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="290">
   <si>
     <t>#</t>
   </si>
@@ -885,6 +885,18 @@
   </si>
   <si>
     <t>LCSC</t>
+  </si>
+  <si>
+    <t>Speaker</t>
+  </si>
+  <si>
+    <t>8 Ohms - 5 Watts</t>
+  </si>
+  <si>
+    <t>FS40DS0850-H18.8</t>
+  </si>
+  <si>
+    <t>FUET</t>
   </si>
 </sst>
 </file>
@@ -2111,7 +2123,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K65"/>
+  <dimension ref="A1:K66"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="3.14285714285714" style="1" customWidth="1"/>
@@ -3360,7 +3372,7 @@
       </c>
       <c r="K39" s="9"/>
     </row>
-    <row r="40" spans="1:11">
+    <row r="40" ht="15.75" spans="1:11">
       <c r="A40" s="2"/>
       <c r="B40" s="7">
         <f t="shared" si="0"/>
@@ -3392,7 +3404,7 @@
       </c>
       <c r="K40" s="11"/>
     </row>
-    <row r="41" spans="1:11">
+    <row r="41" ht="15.75" spans="1:11">
       <c r="A41" s="2"/>
       <c r="B41" s="7">
         <f t="shared" si="0"/>
@@ -3424,7 +3436,7 @@
       </c>
       <c r="K41" s="20"/>
     </row>
-    <row r="42" spans="1:11">
+    <row r="42" ht="15.75" spans="1:11">
       <c r="A42" s="2"/>
       <c r="B42" s="7">
         <f t="shared" si="0"/>
@@ -4199,6 +4211,36 @@
       <c r="K65" s="23" t="s">
         <v>285</v>
       </c>
+    </row>
+    <row r="66" ht="44" customHeight="1" spans="2:11">
+      <c r="B66" s="15">
+        <v>64</v>
+      </c>
+      <c r="C66" s="18" t="s">
+        <v>286</v>
+      </c>
+      <c r="D66" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="E66" s="22" t="s">
+        <v>287</v>
+      </c>
+      <c r="F66" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="G66" s="22" t="s">
+        <v>288</v>
+      </c>
+      <c r="H66" s="22" t="s">
+        <v>289</v>
+      </c>
+      <c r="I66" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="J66" s="22">
+        <v>1</v>
+      </c>
+      <c r="K66" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>